<commit_message>
update bill page -5570663976
</commit_message>
<xml_diff>
--- a/bills/huixinjiqiren/-5570663976/2f51b32dbd10be530766037e3aafda2a0cabe66a37e0289074ce7a7a9f114a35/bill-2026-09-17.xlsx
+++ b/bills/huixinjiqiren/-5570663976/2f51b32dbd10be530766037e3aafda2a0cabe66a37e0289074ce7a7a9f114a35/bill-2026-09-17.xlsx
@@ -72,186 +72,144 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>09/17 18:20:33</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>70000</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>7.8</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>8974.36</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>xinhui9</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="6"/>
+    <row r="5"/>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>代付</t>
+        </is>
+      </c>
+    </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>代付</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
           <t>时间</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>金额</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>费率</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>汇率</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>结算</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>标记人</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>操作人</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
     </row>
-    <row r="9"/>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>下发</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>下发</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
           <t>时间</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>金额</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>标记人</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>操作人</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
     </row>
-    <row r="12"/>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>总计</t>
+        </is>
+      </c>
+    </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>总计</t>
+          <t>总入款</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>总入款</t>
+          <t>应下发</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>70000</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>应下发</t>
+          <t>已下发</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>8974.36</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>已下发</t>
+          <t>未下发</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
           <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>未下发</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>8974.36</t>
         </is>
       </c>
     </row>

</xml_diff>